<commit_message>
#1071 generate zengin result columns dynamically
</commit_message>
<xml_diff>
--- a/app/views/zengin_payments/excels/zengin_results.xlsx
+++ b/app/views/zengin_payments/excels/zengin_results.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\temp\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AB3E396C-4F3D-4018-8D5C-89BCA59C7FD8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4CA6941D-76ED-4886-9201-2B4593A77758}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="42480" yWindow="4330" windowWidth="28800" windowHeight="15370" xr2:uid="{64077235-3348-4162-8948-A6FF4FD43BE3}"/>
+    <workbookView xWindow="3040" yWindow="3040" windowWidth="28800" windowHeight="15370" xr2:uid="{64077235-3348-4162-8948-A6FF4FD43BE3}"/>
   </bookViews>
   <sheets>
     <sheet name="作業者" sheetId="2" r:id="rId1"/>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="20">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="8">
   <si>
     <t>世帯番号</t>
     <rPh sb="0" eb="2">
@@ -95,126 +95,6 @@
   </si>
   <si>
     <t>明細金額1</t>
-    <rPh sb="0" eb="2">
-      <t>メイサイ</t>
-    </rPh>
-    <rPh sb="2" eb="4">
-      <t>キンガク</t>
-    </rPh>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>明細名2</t>
-    <rPh sb="0" eb="2">
-      <t>メイサイ</t>
-    </rPh>
-    <rPh sb="2" eb="3">
-      <t>メイ</t>
-    </rPh>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>明細金額2</t>
-    <rPh sb="0" eb="2">
-      <t>メイサイ</t>
-    </rPh>
-    <rPh sb="2" eb="4">
-      <t>キンガク</t>
-    </rPh>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>明細名3</t>
-    <rPh sb="0" eb="2">
-      <t>メイサイ</t>
-    </rPh>
-    <rPh sb="2" eb="3">
-      <t>メイ</t>
-    </rPh>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>明細金額3</t>
-    <rPh sb="0" eb="2">
-      <t>メイサイ</t>
-    </rPh>
-    <rPh sb="2" eb="4">
-      <t>キンガク</t>
-    </rPh>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>明細名4</t>
-    <rPh sb="0" eb="2">
-      <t>メイサイ</t>
-    </rPh>
-    <rPh sb="2" eb="3">
-      <t>メイ</t>
-    </rPh>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>明細金額4</t>
-    <rPh sb="0" eb="2">
-      <t>メイサイ</t>
-    </rPh>
-    <rPh sb="2" eb="4">
-      <t>キンガク</t>
-    </rPh>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>明細名5</t>
-    <rPh sb="0" eb="2">
-      <t>メイサイ</t>
-    </rPh>
-    <rPh sb="2" eb="3">
-      <t>メイ</t>
-    </rPh>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>明細金額5</t>
-    <rPh sb="0" eb="2">
-      <t>メイサイ</t>
-    </rPh>
-    <rPh sb="2" eb="4">
-      <t>キンガク</t>
-    </rPh>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>明細名6</t>
-    <rPh sb="0" eb="2">
-      <t>メイサイ</t>
-    </rPh>
-    <rPh sb="2" eb="3">
-      <t>メイ</t>
-    </rPh>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>明細金額6</t>
-    <rPh sb="0" eb="2">
-      <t>メイサイ</t>
-    </rPh>
-    <rPh sb="2" eb="4">
-      <t>キンガク</t>
-    </rPh>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>明細名7</t>
-    <rPh sb="0" eb="2">
-      <t>メイサイ</t>
-    </rPh>
-    <rPh sb="2" eb="3">
-      <t>メイ</t>
-    </rPh>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>明細金額7</t>
     <rPh sb="0" eb="2">
       <t>メイサイ</t>
     </rPh>
@@ -629,7 +509,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B16B55BD-AB1E-4B8D-8B67-3A0A036B3EC1}">
-  <dimension ref="A1:T1"/>
+  <dimension ref="A1:H1"/>
   <sheetFormatPr defaultRowHeight="18" x14ac:dyDescent="0.55000000000000004"/>
   <cols>
     <col min="3" max="3" width="8.6640625" style="5"/>
@@ -637,21 +517,9 @@
     <col min="6" max="6" width="8.6640625" style="3"/>
     <col min="7" max="7" width="7.6640625" style="5" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="9.5" style="3" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="7.6640625" style="5" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="9.5" style="3" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="7.6640625" style="5" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="9.5" style="3" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="7.6640625" style="5" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="9.5" style="3" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="7.6640625" style="5" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="9.5" style="3" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="7.6640625" style="5" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="9.5" style="3" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="7.6640625" style="5" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="9.5" style="3" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:20" x14ac:dyDescent="0.55000000000000004">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.55000000000000004">
       <c r="A1" s="1" t="s">
         <v>4</v>
       </c>
@@ -675,42 +543,6 @@
       </c>
       <c r="H1" s="2" t="s">
         <v>7</v>
-      </c>
-      <c r="I1" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="J1" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="K1" s="4" t="s">
-        <v>10</v>
-      </c>
-      <c r="L1" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="M1" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="N1" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="O1" s="4" t="s">
-        <v>14</v>
-      </c>
-      <c r="P1" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="Q1" s="4" t="s">
-        <v>16</v>
-      </c>
-      <c r="R1" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="S1" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="T1" s="2" t="s">
-        <v>19</v>
       </c>
     </row>
   </sheetData>

</xml_diff>